<commit_message>
Terrain : Honotel/HappyCulture (Étoile Saint-Ferdinand) — cibles siège, prochaine tournée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EE1QdXe6TA6RPfxWLeZJgk
</commit_message>
<xml_diff>
--- a/prospection/Prospection-physique.xlsx
+++ b/prospection/Prospection-physique.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -695,6 +695,83 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hôtel Étoile Saint-Ferdinand by HappyCulture (4★, 42 ch.)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>36 rue Saint-Ferdinand, 75017 Paris</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>La réception</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Siège Honotel (le directeur de l'hôtel ne décide pas) : Antoine Foujols, directeur des opérations</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pas de nom ni de mail donnés sur place. Siège : 18 rue Treilhard 75008 · 01 72 32 20 63 · afoujols@happyculture.com (déduit)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Booking 9,3/10</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Réceptionniste IA (pics d'appels pendant les salons, multilingue) + harmonisation des outils, audit pilote gratuit</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Passage à la réception, refus de transmettre le contact</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Approche du siège (Foujols / Le Pogam) + revoir l'hôtel lors de la prochaine tournée</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Siège à contacter</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Terrain : Hôtel Belfast — mail + analyse envoyés, demande de RDV
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EE1QdXe6TA6RPfxWLeZJgk
</commit_message>
<xml_diff>
--- a/prospection/Prospection-physique.xlsx
+++ b/prospection/Prospection-physique.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -772,6 +772,83 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hôtel Belfast (4★, 54 ch.)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10 avenue Carnot, 75017 Paris</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>David (accueil)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Direction (manager signant « Benoit Z. » sur TripAdvisor, à confirmer)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>infos@hotelbelfastparis.com · 01 43 80 12 10</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>TripAdvisor 3,9/5 (249 avis), Kayak 7,9/10 : petit-déj, bruit, chambres datées, service variable</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Réceptionniste IA 24h/24, connexion des logiciels, messages avant/après séjour — env. 48 000 €/an</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Mail + analyse PDF envoyés le 27/10 à 18h21</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RDV audit proposé jeu. 5/11 ou ven. 6/11 à 15 h</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Lun. 2/11 (relance si pas de réponse)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Mail envoyé</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>